<commit_message>
-fixed loop in start dating
</commit_message>
<xml_diff>
--- a/Sharedpointrequest/CurrentlyRunningItem.xlsx
+++ b/Sharedpointrequest/CurrentlyRunningItem.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Public\RPA Folders\Migration\Fusion_ICRules\Sharedpointrequest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5BE4DEF-33F9-4987-85CF-D7EA9D2305E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0620E0-1B89-49D2-9DC0-52FA2F8984F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3210" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="4245" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -30,10 +30,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>